<commit_message>
DB 업데이트 (2026. 6. 30. 오후 3:48:47)
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEBFDD9-BD41-458C-A6E7-7D2203B9B463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB58472-007A-4448-8B56-B157E6200D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24012" yWindow="1488" windowWidth="23016" windowHeight="13656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26820" yWindow="1308" windowWidth="23016" windowHeight="13656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="171">
   <si>
     <t>425-81-02924</t>
   </si>
@@ -541,6 +541,15 @@
   </si>
   <si>
     <t>세한국제1221010</t>
+  </si>
+  <si>
+    <t>308-86-03448</t>
+  </si>
+  <si>
+    <t>주식회사 제이지디글로벌</t>
+  </si>
+  <si>
+    <t>제이지디1251011</t>
   </si>
 </sst>
 </file>
@@ -989,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6138A4-676B-44A6-82D7-1ADA43310F48}">
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1784,6 +1793,20 @@
         <v>46203</v>
       </c>
     </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>168</v>
+      </c>
+      <c r="B56" t="s">
+        <v>169</v>
+      </c>
+      <c r="C56" t="s">
+        <v>170</v>
+      </c>
+      <c r="G56" s="7">
+        <v>46203</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:B1048576">

</xml_diff>

<commit_message>
DB 업데이트 (2026. 6. 30. 오후 3:54:08)
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB58472-007A-4448-8B56-B157E6200D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D42EA567-53A8-41FB-B3C0-C397473A42FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26820" yWindow="1308" windowWidth="23016" windowHeight="13656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2412" yWindow="17172" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="189">
   <si>
     <t>425-81-02924</t>
   </si>
@@ -550,6 +550,60 @@
   </si>
   <si>
     <t>제이지디1251011</t>
+  </si>
+  <si>
+    <t>라워스</t>
+  </si>
+  <si>
+    <t>155-39-01347</t>
+  </si>
+  <si>
+    <t>라워스**5241014</t>
+  </si>
+  <si>
+    <t>로비엔트</t>
+  </si>
+  <si>
+    <t>775-05-03877</t>
+  </si>
+  <si>
+    <t>로비엔트5261019</t>
+  </si>
+  <si>
+    <t>스카이미너리즈</t>
+  </si>
+  <si>
+    <t>819-08-02465</t>
+  </si>
+  <si>
+    <t>스카이미5231013</t>
+  </si>
+  <si>
+    <t>유한회사 엘민커머스</t>
+  </si>
+  <si>
+    <t>829-88-03051</t>
+  </si>
+  <si>
+    <t>엘민커머1241017</t>
+  </si>
+  <si>
+    <t>731-02-03686</t>
+  </si>
+  <si>
+    <t>라비앙하우스</t>
+  </si>
+  <si>
+    <t>라비앙하5251015</t>
+  </si>
+  <si>
+    <t>589-19-02503</t>
+  </si>
+  <si>
+    <t>쓸리보</t>
+  </si>
+  <si>
+    <t>쓸리보**5251019</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1052,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6138A4-676B-44A6-82D7-1ADA43310F48}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1807,6 +1861,90 @@
         <v>46203</v>
       </c>
     </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A57" t="s">
+        <v>172</v>
+      </c>
+      <c r="B57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C57" t="s">
+        <v>173</v>
+      </c>
+      <c r="G57" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>175</v>
+      </c>
+      <c r="B58" t="s">
+        <v>174</v>
+      </c>
+      <c r="C58" t="s">
+        <v>176</v>
+      </c>
+      <c r="G58" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A59" t="s">
+        <v>178</v>
+      </c>
+      <c r="B59" t="s">
+        <v>177</v>
+      </c>
+      <c r="C59" t="s">
+        <v>179</v>
+      </c>
+      <c r="G59" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A60" t="s">
+        <v>181</v>
+      </c>
+      <c r="B60" t="s">
+        <v>180</v>
+      </c>
+      <c r="C60" t="s">
+        <v>182</v>
+      </c>
+      <c r="G60" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A61" t="s">
+        <v>183</v>
+      </c>
+      <c r="B61" t="s">
+        <v>184</v>
+      </c>
+      <c r="C61" t="s">
+        <v>185</v>
+      </c>
+      <c r="G61" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>186</v>
+      </c>
+      <c r="B62" t="s">
+        <v>187</v>
+      </c>
+      <c r="C62" t="s">
+        <v>188</v>
+      </c>
+      <c r="G62" s="7">
+        <v>46203</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:B1048576">

</xml_diff>

<commit_message>
DB 업데이트 (2026. 6. 30. 오후 4:21:59)
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D42EA567-53A8-41FB-B3C0-C397473A42FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4662C168-8AF3-4EE6-B872-DD16A14C26C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2412" yWindow="17172" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="204">
   <si>
     <t>425-81-02924</t>
   </si>
@@ -604,6 +604,51 @@
   </si>
   <si>
     <t>쓸리보**5251019</t>
+  </si>
+  <si>
+    <t>571-81-04069</t>
+  </si>
+  <si>
+    <t>오로라링크 유한회사</t>
+  </si>
+  <si>
+    <t>오로라링1261019</t>
+  </si>
+  <si>
+    <t>344-13-02645</t>
+  </si>
+  <si>
+    <t>모모타로</t>
+  </si>
+  <si>
+    <t>모모타로5231012</t>
+  </si>
+  <si>
+    <t>하임하이</t>
+  </si>
+  <si>
+    <t>343-16-01760</t>
+  </si>
+  <si>
+    <t>하임하이5221012</t>
+  </si>
+  <si>
+    <t>104-34-15402</t>
+  </si>
+  <si>
+    <t>엠티</t>
+  </si>
+  <si>
+    <t>엠티****5231010</t>
+  </si>
+  <si>
+    <t>그린홈컴퍼니</t>
+  </si>
+  <si>
+    <t>801-03-03153</t>
+  </si>
+  <si>
+    <t>그린홈컴5231012</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6138A4-676B-44A6-82D7-1ADA43310F48}">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1945,6 +1990,76 @@
         <v>46203</v>
       </c>
     </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A63" t="s">
+        <v>189</v>
+      </c>
+      <c r="B63" t="s">
+        <v>190</v>
+      </c>
+      <c r="C63" t="s">
+        <v>191</v>
+      </c>
+      <c r="G63" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A64" t="s">
+        <v>192</v>
+      </c>
+      <c r="B64" t="s">
+        <v>193</v>
+      </c>
+      <c r="C64" t="s">
+        <v>194</v>
+      </c>
+      <c r="G64" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A65" t="s">
+        <v>196</v>
+      </c>
+      <c r="B65" t="s">
+        <v>195</v>
+      </c>
+      <c r="C65" t="s">
+        <v>197</v>
+      </c>
+      <c r="G65" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A66" t="s">
+        <v>198</v>
+      </c>
+      <c r="B66" t="s">
+        <v>199</v>
+      </c>
+      <c r="C66" t="s">
+        <v>200</v>
+      </c>
+      <c r="G66" s="7">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A67" t="s">
+        <v>202</v>
+      </c>
+      <c r="B67" t="s">
+        <v>201</v>
+      </c>
+      <c r="C67" t="s">
+        <v>203</v>
+      </c>
+      <c r="G67" s="7">
+        <v>46203</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:B1048576">

</xml_diff>

<commit_message>
DB 업데이트 (2026. 7. 10. 오전 10:08:08)
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7ABB26-C60D-4450-8D89-60F1BFE832B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227B1389-FE07-4A64-B206-C521D927C583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28284" yWindow="768" windowWidth="26376" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20052" yWindow="216" windowWidth="26376" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="1939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2374" uniqueCount="1947">
   <si>
     <t>425-81-02924</t>
   </si>
@@ -6246,13 +6246,43 @@
   <si>
     <t>08717</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>791-12-02771</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>신미우역</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JIN MEIHONG</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010-6618-8331</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>momokim331@naver.com</t>
+  </si>
+  <si>
+    <t>22006</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>인천광역시 연수구 센트럴로 313, 비동 2409호 12-9호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>신미무역5241015</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6334,14 +6364,6 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -6389,9 +6411,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -6486,13 +6507,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -6850,7 +6868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6138A4-676B-44A6-82D7-1ADA43310F48}">
-  <dimension ref="A1:K280"/>
+  <dimension ref="A1:K281"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -15371,6 +15389,35 @@
         <v>1936</v>
       </c>
     </row>
+    <row r="281" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A281" s="32" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B281" t="s">
+        <v>1940</v>
+      </c>
+      <c r="C281" t="s">
+        <v>1946</v>
+      </c>
+      <c r="D281" s="6" t="s">
+        <v>1941</v>
+      </c>
+      <c r="E281" s="6" t="s">
+        <v>1942</v>
+      </c>
+      <c r="F281" s="6" t="s">
+        <v>1943</v>
+      </c>
+      <c r="G281" s="2">
+        <v>46213</v>
+      </c>
+      <c r="H281" s="9" t="s">
+        <v>1944</v>
+      </c>
+      <c r="I281" t="s">
+        <v>1945</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:B1048576">
@@ -15379,9 +15426,6 @@
   <conditionalFormatting sqref="I1:I1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
-  <hyperlinks>
-    <hyperlink ref="F280" r:id="rId1" xr:uid="{5B12B451-33AF-4080-AE37-8D2C8E07BC51}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
DB 업데이트 (2026. 7. 10. 오전 10:16:04)
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227B1389-FE07-4A64-B206-C521D927C583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9464E5EF-64C0-429F-B598-6202AD575E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20052" yWindow="216" windowWidth="26376" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-29952" yWindow="768" windowWidth="26376" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2374" uniqueCount="1947">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2382" uniqueCount="1955">
   <si>
     <t>425-81-02924</t>
   </si>
@@ -6276,6 +6276,38 @@
   </si>
   <si>
     <t>신미무역5241015</t>
+  </si>
+  <si>
+    <t>08371</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 구로구 디지털로31길 119, 201동 1003호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010-5678-9899</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>qthyzq123@naver.com</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LIU CHUNYING</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>434-13-02759</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>라엔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>라엔****5251017</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -6868,7 +6900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6138A4-676B-44A6-82D7-1ADA43310F48}">
-  <dimension ref="A1:K281"/>
+  <dimension ref="A1:K282"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -15376,7 +15408,7 @@
       <c r="E280" s="6" t="s">
         <v>1934</v>
       </c>
-      <c r="F280" s="40" t="s">
+      <c r="F280" t="s">
         <v>1935</v>
       </c>
       <c r="G280" s="2">
@@ -15416,6 +15448,35 @@
       </c>
       <c r="I281" t="s">
         <v>1945</v>
+      </c>
+    </row>
+    <row r="282" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A282" s="32" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B282" t="s">
+        <v>1953</v>
+      </c>
+      <c r="C282" t="s">
+        <v>1954</v>
+      </c>
+      <c r="D282" s="6" t="s">
+        <v>1951</v>
+      </c>
+      <c r="E282" s="6" t="s">
+        <v>1949</v>
+      </c>
+      <c r="F282" s="40" t="s">
+        <v>1950</v>
+      </c>
+      <c r="G282" s="2">
+        <v>46213</v>
+      </c>
+      <c r="H282" s="9" t="s">
+        <v>1947</v>
+      </c>
+      <c r="I282" t="s">
+        <v>1948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DB 업데이트 (2026. 7. 14. 오후 1:41:05)
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B5C9E4-B683-4B27-9D5A-12D8613C8EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB1931A-71A7-4108-8EBD-7E0E32ABCB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29088" yWindow="252" windowWidth="26376" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28164" yWindow="360" windowWidth="26376" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2382" uniqueCount="2124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="2657">
   <si>
     <t>425-81-02924</t>
   </si>
@@ -6817,6 +6817,1605 @@
   </si>
   <si>
     <t>블루밍로1251013</t>
+  </si>
+  <si>
+    <t>유한회사 비즈랜드코리아</t>
+  </si>
+  <si>
+    <t>비즈랜드1241013</t>
+  </si>
+  <si>
+    <t>WANG HUAXIAO</t>
+  </si>
+  <si>
+    <t>01088721688</t>
+  </si>
+  <si>
+    <t>beadslandshop@163.com</t>
+  </si>
+  <si>
+    <t>경기도 화성시 동탄중심상가2길 26-15(반송동)지성프라자</t>
+  </si>
+  <si>
+    <t>전자상거래</t>
+  </si>
+  <si>
+    <t>전자상거래 외</t>
+  </si>
+  <si>
+    <t>이매력</t>
+  </si>
+  <si>
+    <t>이매력**5241013</t>
+  </si>
+  <si>
+    <t>LI YINGHAI</t>
+  </si>
+  <si>
+    <t>01076886588</t>
+  </si>
+  <si>
+    <t>liyinghai512@naver.com</t>
+  </si>
+  <si>
+    <t>17921</t>
+  </si>
+  <si>
+    <t>경기도 평택시 원평로75번길 39(평택동)</t>
+  </si>
+  <si>
+    <t>피카루샵 유한회사</t>
+  </si>
+  <si>
+    <t>피카루샵1261017</t>
+  </si>
+  <si>
+    <t>LIU SHIYANG</t>
+  </si>
+  <si>
+    <t>010-5722-8444</t>
+  </si>
+  <si>
+    <t>lshy202603@163.com</t>
+  </si>
+  <si>
+    <t>08536</t>
+  </si>
+  <si>
+    <t>서울특별시 금천구 시흥대로152길 11-31 (독산동)3층303-비49호</t>
+  </si>
+  <si>
+    <t>다우기업 (주)</t>
+  </si>
+  <si>
+    <t>다우기업1921018</t>
+  </si>
+  <si>
+    <t>전향진</t>
+  </si>
+  <si>
+    <t>010-3601-1375</t>
+  </si>
+  <si>
+    <t>dawoo2626@hanmail.net</t>
+  </si>
+  <si>
+    <t>58256</t>
+  </si>
+  <si>
+    <t>전라남도 나주시 중앙로 45 (성북동)</t>
+  </si>
+  <si>
+    <t>건설업</t>
+  </si>
+  <si>
+    <t>냉난방위생배관설비공</t>
+  </si>
+  <si>
+    <t>굿앱더몰</t>
+  </si>
+  <si>
+    <t>굿앱더몰5221010</t>
+  </si>
+  <si>
+    <t>박주연</t>
+  </si>
+  <si>
+    <t>01051988982</t>
+  </si>
+  <si>
+    <t>qufrb16@naver.com</t>
+  </si>
+  <si>
+    <t>08814</t>
+  </si>
+  <si>
+    <t>서울특별시 관악구 신림로 99(신림동)센터스퀘어 서울대점</t>
+  </si>
+  <si>
+    <t>월간리빙</t>
+  </si>
+  <si>
+    <t>월간리빙5221013</t>
+  </si>
+  <si>
+    <t>심재원</t>
+  </si>
+  <si>
+    <t>01057497765</t>
+  </si>
+  <si>
+    <t>monthliv@naver.com</t>
+  </si>
+  <si>
+    <t>12913</t>
+  </si>
+  <si>
+    <t>경기도 하남시 미사강변중앙로 208(망월동)부강타워</t>
+  </si>
+  <si>
+    <t>엠에이치케미칼</t>
+  </si>
+  <si>
+    <t>엠에이치522C018</t>
+  </si>
+  <si>
+    <t>이규배</t>
+  </si>
+  <si>
+    <t>01054793509</t>
+  </si>
+  <si>
+    <t>Kblee@mhchem1.com</t>
+  </si>
+  <si>
+    <t>18126</t>
+  </si>
+  <si>
+    <t>경기도 오산시 수목원로88번길 35 (가수동)</t>
+  </si>
+  <si>
+    <t>제조업 외</t>
+  </si>
+  <si>
+    <t>기타화학약품</t>
+  </si>
+  <si>
+    <t>주식회사 데이무드</t>
+  </si>
+  <si>
+    <t>데이무드1232015</t>
+  </si>
+  <si>
+    <t>박영선</t>
+  </si>
+  <si>
+    <t>01022982289</t>
+  </si>
+  <si>
+    <t>oppo2022@naver.com</t>
+  </si>
+  <si>
+    <t>46557</t>
+  </si>
+  <si>
+    <t>부산광역시 북구 상학로 36 (만덕동, 이편한세상 금정산) 201동 1004호</t>
+  </si>
+  <si>
+    <t>도매및소매업</t>
+  </si>
+  <si>
+    <t>전자상거래소매업</t>
+  </si>
+  <si>
+    <t>포커스포인트 유한회사</t>
+  </si>
+  <si>
+    <t>포커스포1251018</t>
+  </si>
+  <si>
+    <t>NING YAWEN</t>
+  </si>
+  <si>
+    <t>010-7980-0389</t>
+  </si>
+  <si>
+    <t>188862017@qq.com</t>
+  </si>
+  <si>
+    <t>11673</t>
+  </si>
+  <si>
+    <t>경기도 의정부시 둔야로33번길 9(의정부동)덕암오피스텔</t>
+  </si>
+  <si>
+    <t>도소매업</t>
+  </si>
+  <si>
+    <t>센리</t>
+  </si>
+  <si>
+    <t>센리****5242018</t>
+  </si>
+  <si>
+    <t>이정민</t>
+  </si>
+  <si>
+    <t>01076302141</t>
+  </si>
+  <si>
+    <t>cs_01@cenli.co.kr</t>
+  </si>
+  <si>
+    <t>41922</t>
+  </si>
+  <si>
+    <t>대구광역시 중구 달성로 123(달성동)달성파크푸르지오힐스테이트</t>
+  </si>
+  <si>
+    <t>어드레스팔공팔</t>
+  </si>
+  <si>
+    <t>어드레스5162010</t>
+  </si>
+  <si>
+    <t>이자원</t>
+  </si>
+  <si>
+    <t>010-5036-8089</t>
+  </si>
+  <si>
+    <t>address808@naver.com</t>
+  </si>
+  <si>
+    <t>18403</t>
+  </si>
+  <si>
+    <t>경기도 화성시 병점구 병점동로 78 (병점동)</t>
+  </si>
+  <si>
+    <t>소매업</t>
+  </si>
+  <si>
+    <t>의류 외</t>
+  </si>
+  <si>
+    <t>(주)엔시스</t>
+  </si>
+  <si>
+    <t>엔시스**1061012</t>
+  </si>
+  <si>
+    <t>진승언</t>
+  </si>
+  <si>
+    <t>041-568-7222</t>
+  </si>
+  <si>
+    <t>yjhwang@n-sys.co.kr</t>
+  </si>
+  <si>
+    <t>31418</t>
+  </si>
+  <si>
+    <t>충청남도 아산시 음봉면 스마트산단3로 18</t>
+  </si>
+  <si>
+    <t>제조 외</t>
+  </si>
+  <si>
+    <t>자동화설비제작및가공</t>
+  </si>
+  <si>
+    <t>젠올데이</t>
+  </si>
+  <si>
+    <t>젠올데이5241010</t>
+  </si>
+  <si>
+    <t>김은호</t>
+  </si>
+  <si>
+    <t>01048461415</t>
+  </si>
+  <si>
+    <t>euniory@naver.com</t>
+  </si>
+  <si>
+    <t>15476</t>
+  </si>
+  <si>
+    <t>경기도 안산시 단원구 광덕서로 54 (고잔동)</t>
+  </si>
+  <si>
+    <t>혜준스토어</t>
+  </si>
+  <si>
+    <t>혜준스토5231015</t>
+  </si>
+  <si>
+    <t>최혜림</t>
+  </si>
+  <si>
+    <t>010-7313-8356</t>
+  </si>
+  <si>
+    <t>en2zz@naver.com</t>
+  </si>
+  <si>
+    <t>경기도 파주시 소리천로 203 (와동동, 가람마을14단지)1402동 1605호</t>
+  </si>
+  <si>
+    <t>피즈모 유한회사</t>
+  </si>
+  <si>
+    <t>피즈모**1251015</t>
+  </si>
+  <si>
+    <t>WANG QIN</t>
+  </si>
+  <si>
+    <t>01082916183</t>
+  </si>
+  <si>
+    <t>1527303592@qq.com</t>
+  </si>
+  <si>
+    <t>부산광역시 강서구 신호삼로 66(신호동)삼성빌딩</t>
+  </si>
+  <si>
+    <t>글로벌픽</t>
+  </si>
+  <si>
+    <t>글로벌픽5181011</t>
+  </si>
+  <si>
+    <t>노복순</t>
+  </si>
+  <si>
+    <t>01076050760</t>
+  </si>
+  <si>
+    <t>bubbleman24@naver.com</t>
+  </si>
+  <si>
+    <t>58115</t>
+  </si>
+  <si>
+    <t>전라남도 화순군 화순읍 용곡3길 106</t>
+  </si>
+  <si>
+    <t>서비스 외</t>
+  </si>
+  <si>
+    <t>무인빨래방 외</t>
+  </si>
+  <si>
+    <t>주식회사 하이올렛</t>
+  </si>
+  <si>
+    <t>하이올렛1221019</t>
+  </si>
+  <si>
+    <t>김진아</t>
+  </si>
+  <si>
+    <t>01080626455</t>
+  </si>
+  <si>
+    <t>hhiolet@naver.com</t>
+  </si>
+  <si>
+    <t>인천광역시 연수구 송도미래로 30, E동 2310호</t>
+  </si>
+  <si>
+    <t>전자상거래소매업외</t>
+  </si>
+  <si>
+    <t>모두바잉</t>
+  </si>
+  <si>
+    <t>모두바잉5221015</t>
+  </si>
+  <si>
+    <t>한은정</t>
+  </si>
+  <si>
+    <t>01099968433</t>
+  </si>
+  <si>
+    <t>hej2220@naver.com</t>
+  </si>
+  <si>
+    <t>05275</t>
+  </si>
+  <si>
+    <t>서울특별시 강동구 상일로 55 (상일동, 고덕자이)118동 403호</t>
+  </si>
+  <si>
+    <t>한민국제화학(주)안성제2공장</t>
+  </si>
+  <si>
+    <t>한민국제1901038</t>
+  </si>
+  <si>
+    <t>나용택</t>
+  </si>
+  <si>
+    <t>010-9034-9467</t>
+  </si>
+  <si>
+    <t>hanminch@daum.net</t>
+  </si>
+  <si>
+    <t>17524</t>
+  </si>
+  <si>
+    <t>경기도 안성시 죽산면 걸미로 363-10</t>
+  </si>
+  <si>
+    <t>제조업</t>
+  </si>
+  <si>
+    <t>유리,복층유리</t>
+  </si>
+  <si>
+    <t>(주)블루건설</t>
+  </si>
+  <si>
+    <t>블루건설1072014</t>
+  </si>
+  <si>
+    <t>박찬우</t>
+  </si>
+  <si>
+    <t>010-3513-2393</t>
+  </si>
+  <si>
+    <t>5553100@naver.com</t>
+  </si>
+  <si>
+    <t>41491</t>
+  </si>
+  <si>
+    <t>대구광역시 북구 문주길 29-9 (금호동)</t>
+  </si>
+  <si>
+    <t>건설업외</t>
+  </si>
+  <si>
+    <t>일반건축외</t>
+  </si>
+  <si>
+    <t>마녀홀릭</t>
+  </si>
+  <si>
+    <t>마녀홀릭5231018</t>
+  </si>
+  <si>
+    <t>하리나</t>
+  </si>
+  <si>
+    <t>01050956180</t>
+  </si>
+  <si>
+    <t>rina1082@naver.com</t>
+  </si>
+  <si>
+    <t>15010</t>
+  </si>
+  <si>
+    <t>경기도 시흥시 배곧4로 106-25(배곧동)호반베르디움 센트로하임아파트</t>
+  </si>
+  <si>
+    <t>아온</t>
+  </si>
+  <si>
+    <t>아온****5211013</t>
+  </si>
+  <si>
+    <t>임상현</t>
+  </si>
+  <si>
+    <t>01096085548</t>
+  </si>
+  <si>
+    <t>dqd2134@naver.com</t>
+  </si>
+  <si>
+    <t>03601</t>
+  </si>
+  <si>
+    <t>서울특별시 서대문구 홍은중앙로 128-13(홍은동)</t>
+  </si>
+  <si>
+    <t>해외직구대행업 외</t>
+  </si>
+  <si>
+    <t>주식회사 케이씨씨실리콘 전주</t>
+  </si>
+  <si>
+    <t>케이씨씨1202035</t>
+  </si>
+  <si>
+    <t>송영근</t>
+  </si>
+  <si>
+    <t>55321</t>
+  </si>
+  <si>
+    <t>전북특별자치도 완주군 봉동읍 과학로 801</t>
+  </si>
+  <si>
+    <t>화합물 및 화학제품</t>
+  </si>
+  <si>
+    <t>주식회사 케이씨씨실리콘 영업</t>
+  </si>
+  <si>
+    <t>케이씨씨1202028</t>
+  </si>
+  <si>
+    <t>02-3495-2115</t>
+  </si>
+  <si>
+    <t>06608</t>
+  </si>
+  <si>
+    <t>서울특별시 서초구 사평대로 344 (서초동)</t>
+  </si>
+  <si>
+    <t>화학물질 및 화학제품</t>
+  </si>
+  <si>
+    <t>케이앤피컴퍼니</t>
+  </si>
+  <si>
+    <t>케이앤피5222019</t>
+  </si>
+  <si>
+    <t>김일</t>
+  </si>
+  <si>
+    <t>01063735668</t>
+  </si>
+  <si>
+    <t>kimil1107@naver.com</t>
+  </si>
+  <si>
+    <t>08314</t>
+  </si>
+  <si>
+    <t>서울특별시 구로구 구로동로8길 50 (구로동)</t>
+  </si>
+  <si>
+    <t>소매 외</t>
+  </si>
+  <si>
+    <t>주식회사이레건설산업</t>
+  </si>
+  <si>
+    <t>이레건설1081017</t>
+  </si>
+  <si>
+    <t>정민혁</t>
+  </si>
+  <si>
+    <t>01032497934</t>
+  </si>
+  <si>
+    <t>jyyoon@ereenc.com</t>
+  </si>
+  <si>
+    <t>13002</t>
+  </si>
+  <si>
+    <t>경기도 하남시 감일로72번길 19 (감일동)</t>
+  </si>
+  <si>
+    <t>종합건설 외</t>
+  </si>
+  <si>
+    <t>셀리온 유한회사</t>
+  </si>
+  <si>
+    <t>셀리온**1251014</t>
+  </si>
+  <si>
+    <t>YU LANHAI</t>
+  </si>
+  <si>
+    <t>01073956352</t>
+  </si>
+  <si>
+    <t>404836164@qq.com</t>
+  </si>
+  <si>
+    <t>충청북도 청주시 상당구 성안로74번길 18-1 (남문로1가)</t>
+  </si>
+  <si>
+    <t>전자상거래 소매업 외</t>
+  </si>
+  <si>
+    <t>트리풀마켓</t>
+  </si>
+  <si>
+    <t>트리풀마5251019</t>
+  </si>
+  <si>
+    <t>최아영</t>
+  </si>
+  <si>
+    <t>01038403477</t>
+  </si>
+  <si>
+    <t>trifullmarket@gmail.com</t>
+  </si>
+  <si>
+    <t>29022</t>
+  </si>
+  <si>
+    <t>충청북도 옥천군 동이면 우산로1길 131-8</t>
+  </si>
+  <si>
+    <t>소매업 외</t>
+  </si>
+  <si>
+    <t>명진</t>
+  </si>
+  <si>
+    <t>명진****5081011</t>
+  </si>
+  <si>
+    <t>김주홍</t>
+  </si>
+  <si>
+    <t>01022503800</t>
+  </si>
+  <si>
+    <t>mj5299@naver.com</t>
+  </si>
+  <si>
+    <t>18515</t>
+  </si>
+  <si>
+    <t>경기도 화성시 효행구 정남면 정남동로 33-29</t>
+  </si>
+  <si>
+    <t>LCD,반도체장비,부품</t>
+  </si>
+  <si>
+    <t>(주)유에이아이</t>
+  </si>
+  <si>
+    <t>유에이아1031017</t>
+  </si>
+  <si>
+    <t>노기환</t>
+  </si>
+  <si>
+    <t>01025769650</t>
+  </si>
+  <si>
+    <t>yuna@uai.kr?</t>
+  </si>
+  <si>
+    <t>13516</t>
+  </si>
+  <si>
+    <t>경기도 성남시 분당구 판교로 700 (야탑동)</t>
+  </si>
+  <si>
+    <t>소프트웨어개발및공급</t>
+  </si>
+  <si>
+    <t>엑스마시르트레이딩 유한회사</t>
+  </si>
+  <si>
+    <t>엑스마시1251010</t>
+  </si>
+  <si>
+    <t>QIN WEIWEI</t>
+  </si>
+  <si>
+    <t>07077716872</t>
+  </si>
+  <si>
+    <t>1753625128@qq.com</t>
+  </si>
+  <si>
+    <t>경기도 이천시 향교로 68(창전동)</t>
+  </si>
+  <si>
+    <t>반야월소</t>
+  </si>
+  <si>
+    <t>반야월소5181019</t>
+  </si>
+  <si>
+    <t>황현숙</t>
+  </si>
+  <si>
+    <t>01045337428</t>
+  </si>
+  <si>
+    <t>banyawolso@gmail.com</t>
+  </si>
+  <si>
+    <t>41128</t>
+  </si>
+  <si>
+    <t>대구광역시 동구 반야월북로2길 28, 1층</t>
+  </si>
+  <si>
+    <t>제조업외</t>
+  </si>
+  <si>
+    <t>기타목재가구제조업외</t>
+  </si>
+  <si>
+    <t>인포테크 유한회사</t>
+  </si>
+  <si>
+    <t>인포테크1251019</t>
+  </si>
+  <si>
+    <t>CHEN GEYANG</t>
+  </si>
+  <si>
+    <t>07047321871</t>
+  </si>
+  <si>
+    <t>i6270959@gmail.com</t>
+  </si>
+  <si>
+    <t>경기도 김포시 김포한강9로75번길 22(구래동)</t>
+  </si>
+  <si>
+    <t>스티브잉크 유한회사</t>
+  </si>
+  <si>
+    <t>스티브잉1261019</t>
+  </si>
+  <si>
+    <t>GUO XIANGAN</t>
+  </si>
+  <si>
+    <t>07077329074</t>
+  </si>
+  <si>
+    <t>19940322gxg@gmail.com</t>
+  </si>
+  <si>
+    <t>05043</t>
+  </si>
+  <si>
+    <t>서울특별시 광진구 자양로18길 17 (구의동)</t>
+  </si>
+  <si>
+    <t>청양구기자원예농업협동조합</t>
+  </si>
+  <si>
+    <t>청양구기2941016</t>
+  </si>
+  <si>
+    <t>복영수</t>
+  </si>
+  <si>
+    <t>01062313652</t>
+  </si>
+  <si>
+    <t>cykukija@hanmail.net</t>
+  </si>
+  <si>
+    <t>33332</t>
+  </si>
+  <si>
+    <t>충청남도 청양군 청양읍 칠갑산로4길 28</t>
+  </si>
+  <si>
+    <t>서비스,제조 외</t>
+  </si>
+  <si>
+    <t>위탁,다류 외</t>
+  </si>
+  <si>
+    <t>성선백화점</t>
+  </si>
+  <si>
+    <t>성선백화5251012</t>
+  </si>
+  <si>
+    <t>LI YAJU</t>
+  </si>
+  <si>
+    <t>01084128876</t>
+  </si>
+  <si>
+    <t>ly133334450@163.com</t>
+  </si>
+  <si>
+    <t>05037</t>
+  </si>
+  <si>
+    <t>서울 광진구 광나루로38길 63</t>
+  </si>
+  <si>
+    <t>소매</t>
+  </si>
+  <si>
+    <t>일용잡화</t>
+  </si>
+  <si>
+    <t>(주)노디너리</t>
+  </si>
+  <si>
+    <t>노디너리1201015</t>
+  </si>
+  <si>
+    <t>백문기</t>
+  </si>
+  <si>
+    <t>01022381263</t>
+  </si>
+  <si>
+    <t>sales@nordinary.co.kr</t>
+  </si>
+  <si>
+    <t>18469</t>
+  </si>
+  <si>
+    <t>경기도 화성시 동탄구 동탄첨단산업1로 27 (영천동)</t>
+  </si>
+  <si>
+    <t>화장품 원료 외</t>
+  </si>
+  <si>
+    <t>오성홀딩스 주식회사</t>
+  </si>
+  <si>
+    <t>오성홀딩1211015</t>
+  </si>
+  <si>
+    <t>서일현</t>
+  </si>
+  <si>
+    <t>01031122210</t>
+  </si>
+  <si>
+    <t>finetex77@naver.com</t>
+  </si>
+  <si>
+    <t>22530</t>
+  </si>
+  <si>
+    <t>인천광역시 동구 방축로83번길 23 (송림동)</t>
+  </si>
+  <si>
+    <t>공업자재 외</t>
+  </si>
+  <si>
+    <t>샵큐</t>
+  </si>
+  <si>
+    <t>샵큐****5191018</t>
+  </si>
+  <si>
+    <t>이상범</t>
+  </si>
+  <si>
+    <t>01052416606</t>
+  </si>
+  <si>
+    <t>shopq2@shopq.co.kr</t>
+  </si>
+  <si>
+    <t>12285</t>
+  </si>
+  <si>
+    <t>경기도 남양주시 다산순환로 365(다산동)힐스테이트 다산</t>
+  </si>
+  <si>
+    <t>도매 및 소매업 외</t>
+  </si>
+  <si>
+    <t>키맨</t>
+  </si>
+  <si>
+    <t>키맨****5261019</t>
+  </si>
+  <si>
+    <t>김시현</t>
+  </si>
+  <si>
+    <t>01093188386</t>
+  </si>
+  <si>
+    <t>foremost.keyman@gmail.com</t>
+  </si>
+  <si>
+    <t>10908</t>
+  </si>
+  <si>
+    <t>경기도 파주시 와석순환로 16 (야당동, 롯데캐슬파크타운)</t>
+  </si>
+  <si>
+    <t>업튼</t>
+  </si>
+  <si>
+    <t>업튼****5151014</t>
+  </si>
+  <si>
+    <t>임성건</t>
+  </si>
+  <si>
+    <t>01035827371</t>
+  </si>
+  <si>
+    <t>5827371@naver.com</t>
+  </si>
+  <si>
+    <t>48582</t>
+  </si>
+  <si>
+    <t>부산광역시 남구 용호로159번길 94 (용호동)</t>
+  </si>
+  <si>
+    <t>스포츠의류 외</t>
+  </si>
+  <si>
+    <t>전자상거래업 외</t>
+  </si>
+  <si>
+    <t>페블러스</t>
+  </si>
+  <si>
+    <t>페블러스5171017</t>
+  </si>
+  <si>
+    <t>이승진</t>
+  </si>
+  <si>
+    <t>01034240604</t>
+  </si>
+  <si>
+    <t>fabulous1030@naver.com</t>
+  </si>
+  <si>
+    <t>07264</t>
+  </si>
+  <si>
+    <t>서울특별시 영등포구 영등포로 109</t>
+  </si>
+  <si>
+    <t>주식회사 선진식품</t>
+  </si>
+  <si>
+    <t>선진식품1131019</t>
+  </si>
+  <si>
+    <t>김만제</t>
+  </si>
+  <si>
+    <t>01051330228</t>
+  </si>
+  <si>
+    <t>sunjin0063@hanmail.net</t>
+  </si>
+  <si>
+    <t>18255</t>
+  </si>
+  <si>
+    <t>경기도 화성시 만세구 남양읍 주석로184번길 69</t>
+  </si>
+  <si>
+    <t>순대 외</t>
+  </si>
+  <si>
+    <t>퍼포먼스 메이커</t>
+  </si>
+  <si>
+    <t>퍼포먼스5231012</t>
+  </si>
+  <si>
+    <t>오시훈</t>
+  </si>
+  <si>
+    <t>01092607739</t>
+  </si>
+  <si>
+    <t>sihun950405@gmail.com</t>
+  </si>
+  <si>
+    <t>46981</t>
+  </si>
+  <si>
+    <t>부산광역시 사상구 새벽로 170(감전동)</t>
+  </si>
+  <si>
+    <t>(주)안성내츄럴리조트</t>
+  </si>
+  <si>
+    <t>안성내츄1101017</t>
+  </si>
+  <si>
+    <t>곽숙자</t>
+  </si>
+  <si>
+    <t>01037290774</t>
+  </si>
+  <si>
+    <t>uni0774@naver.com</t>
+  </si>
+  <si>
+    <t>17518</t>
+  </si>
+  <si>
+    <t>경기도 안성시 죽산면 죽양대로 136-16</t>
+  </si>
+  <si>
+    <t>생수 생산업 외</t>
+  </si>
+  <si>
+    <t>천일공작소</t>
+  </si>
+  <si>
+    <t>천일공작5211010</t>
+  </si>
+  <si>
+    <t>양희순</t>
+  </si>
+  <si>
+    <t>01056430523</t>
+  </si>
+  <si>
+    <t>yhs123q@naver.com</t>
+  </si>
+  <si>
+    <t>58509</t>
+  </si>
+  <si>
+    <t>전라남도 무안군 현경면 현해로 816</t>
+  </si>
+  <si>
+    <t>(주)채움가구</t>
+  </si>
+  <si>
+    <t>채움가구1181012</t>
+  </si>
+  <si>
+    <t>김만기</t>
+  </si>
+  <si>
+    <t>01090826887</t>
+  </si>
+  <si>
+    <t>chaeum03@naver.com</t>
+  </si>
+  <si>
+    <t>11160</t>
+  </si>
+  <si>
+    <t>경기도 포천시 삼육사로 2019-32 (선단동)</t>
+  </si>
+  <si>
+    <t>가구 외</t>
+  </si>
+  <si>
+    <t>(주)메디치코리아코스메틱</t>
+  </si>
+  <si>
+    <t>메디치코1141014</t>
+  </si>
+  <si>
+    <t>오정미</t>
+  </si>
+  <si>
+    <t>031-666-3120</t>
+  </si>
+  <si>
+    <t>17749</t>
+  </si>
+  <si>
+    <t>경기도 평택시 동삭로 455-64 (칠괴동)</t>
+  </si>
+  <si>
+    <t>화장품</t>
+  </si>
+  <si>
+    <t>몽디자인</t>
+  </si>
+  <si>
+    <t>몽디자인5191017</t>
+  </si>
+  <si>
+    <t>김상엽</t>
+  </si>
+  <si>
+    <t>01049496344</t>
+  </si>
+  <si>
+    <t>mong2131@naver.com</t>
+  </si>
+  <si>
+    <t>21583</t>
+  </si>
+  <si>
+    <t>인천광역시 남동구 선수촌공원로 30 (구월동)</t>
+  </si>
+  <si>
+    <t>건설업,가구 외</t>
+  </si>
+  <si>
+    <t>실내인테리어,디자인</t>
+  </si>
+  <si>
+    <t>하오셀렉트</t>
+  </si>
+  <si>
+    <t>하오셀렉5251015</t>
+  </si>
+  <si>
+    <t>예민서</t>
+  </si>
+  <si>
+    <t>01084586884</t>
+  </si>
+  <si>
+    <t>y0331252@gmail.com</t>
+  </si>
+  <si>
+    <t>48502</t>
+  </si>
+  <si>
+    <t>부산광역시 남구 유엔로157번가길 75 (대연동)</t>
+  </si>
+  <si>
+    <t>주식회사 와클글로벌</t>
+  </si>
+  <si>
+    <t>와클글로1181016</t>
+  </si>
+  <si>
+    <t>김한용</t>
+  </si>
+  <si>
+    <t>01031467488</t>
+  </si>
+  <si>
+    <t>wacle7478@naver.com</t>
+  </si>
+  <si>
+    <t>10910</t>
+  </si>
+  <si>
+    <t>경기도 파주시 하우4길 26-26 (상지석동)</t>
+  </si>
+  <si>
+    <t>폐수처리장비 외</t>
+  </si>
+  <si>
+    <t>하나비</t>
+  </si>
+  <si>
+    <t>하나비**5261011</t>
+  </si>
+  <si>
+    <t>윤승현</t>
+  </si>
+  <si>
+    <t>01095520968</t>
+  </si>
+  <si>
+    <t>Hanabi.luke.yun@gmail.com</t>
+  </si>
+  <si>
+    <t>04968</t>
+  </si>
+  <si>
+    <t>서울특별시 광진구 아차산로73길 48 (광장동)</t>
+  </si>
+  <si>
+    <t>음식점업</t>
+  </si>
+  <si>
+    <t>카페</t>
+  </si>
+  <si>
+    <t>기억한조각</t>
+  </si>
+  <si>
+    <t>기억한조5211017</t>
+  </si>
+  <si>
+    <t>송사라</t>
+  </si>
+  <si>
+    <t>01084902486</t>
+  </si>
+  <si>
+    <t>sosu0412@naver.com</t>
+  </si>
+  <si>
+    <t>35277</t>
+  </si>
+  <si>
+    <t>대전광역시 서구 신갈마로 161 (갈마동)</t>
+  </si>
+  <si>
+    <t>휴게음식점(레터링케</t>
+  </si>
+  <si>
+    <t>(주)글로우서울</t>
+  </si>
+  <si>
+    <t>글로우서1181015</t>
+  </si>
+  <si>
+    <t>유정수,윤성혁</t>
+  </si>
+  <si>
+    <t>01095175658</t>
+  </si>
+  <si>
+    <t>dmi3302@naver.com</t>
+  </si>
+  <si>
+    <t>04351</t>
+  </si>
+  <si>
+    <t>서울특별시 용산구 이태원로17길 23-8(이태원동)오스카164B</t>
+  </si>
+  <si>
+    <t>식음료 외</t>
+  </si>
+  <si>
+    <t>조소</t>
+  </si>
+  <si>
+    <t>조소****5121017</t>
+  </si>
+  <si>
+    <t>조윤형</t>
+  </si>
+  <si>
+    <t>010-8897-8835</t>
+  </si>
+  <si>
+    <t>hw961016@naver.com</t>
+  </si>
+  <si>
+    <t>03974</t>
+  </si>
+  <si>
+    <t>서울특별시 마포구 연남로13길 31(성산동)동양하우징</t>
+  </si>
+  <si>
+    <t>제조업,임대업</t>
+  </si>
+  <si>
+    <t>공연용소품제조 외</t>
+  </si>
+  <si>
+    <t>와이제이 컴퍼니</t>
+  </si>
+  <si>
+    <t>와이제이520e018</t>
+  </si>
+  <si>
+    <t>최용</t>
+  </si>
+  <si>
+    <t>01034419856</t>
+  </si>
+  <si>
+    <t>cy728@daum.net</t>
+  </si>
+  <si>
+    <t>07635</t>
+  </si>
+  <si>
+    <t>서울특별시 강서구 강서로47길 165 (내발산동)</t>
+  </si>
+  <si>
+    <t>주식회사랩가이드</t>
+  </si>
+  <si>
+    <t>랩가이드1151015</t>
+  </si>
+  <si>
+    <t>정승남</t>
+  </si>
+  <si>
+    <t>01093884574</t>
+  </si>
+  <si>
+    <t>tax@labguide.kr</t>
+  </si>
+  <si>
+    <t>41516</t>
+  </si>
+  <si>
+    <t>대구광역시 북구 유통단지로24길 37 (산격동)</t>
+  </si>
+  <si>
+    <t>과학의료장비판매 외</t>
+  </si>
+  <si>
+    <t>주식회사 신우</t>
+  </si>
+  <si>
+    <t>신우****1251019</t>
+  </si>
+  <si>
+    <t>WANG CHENXU</t>
+  </si>
+  <si>
+    <t>010-7628-8629</t>
+  </si>
+  <si>
+    <t>SHINWOOKR2299@gmail.com</t>
+  </si>
+  <si>
+    <t>12759</t>
+  </si>
+  <si>
+    <t>경기도 광주시 경안로 23 (경안동)</t>
+  </si>
+  <si>
+    <t>세화</t>
+  </si>
+  <si>
+    <t>세화****5221010</t>
+  </si>
+  <si>
+    <t>윤명철</t>
+  </si>
+  <si>
+    <t>01058861666</t>
+  </si>
+  <si>
+    <t>seonhwa0117@gmail.com</t>
+  </si>
+  <si>
+    <t>07318</t>
+  </si>
+  <si>
+    <t>서울특별시 영등포구 영등포로79길 9 (신길동)</t>
+  </si>
+  <si>
+    <t>휴온지엑스스튜디오</t>
+  </si>
+  <si>
+    <t>휴온지엑5261010</t>
+  </si>
+  <si>
+    <t>김다슬</t>
+  </si>
+  <si>
+    <t>01033232583</t>
+  </si>
+  <si>
+    <t>hueon.gx@gmail.com</t>
+  </si>
+  <si>
+    <t>13604</t>
+  </si>
+  <si>
+    <t>경기도 성남시 분당구 불곡로 4 (정자동)</t>
+  </si>
+  <si>
+    <t>서비스업</t>
+  </si>
+  <si>
+    <t>매트운동</t>
+  </si>
+  <si>
+    <t>라비엣</t>
+  </si>
+  <si>
+    <t>라비엣**5251014</t>
+  </si>
+  <si>
+    <t>ZHAO YINGLAN</t>
+  </si>
+  <si>
+    <t>01097911588</t>
+  </si>
+  <si>
+    <t>yeongran87@naver.com</t>
+  </si>
+  <si>
+    <t>22776</t>
+  </si>
+  <si>
+    <t>인천광역시 서해구 봉오대로 270 (가정동, 루원시티2차 SK Leaders VIEW)</t>
+  </si>
+  <si>
+    <t>상품 종합 도매업</t>
+  </si>
+  <si>
+    <t>840-86-03374</t>
+  </si>
+  <si>
+    <t>875-41-01139</t>
+  </si>
+  <si>
+    <t>445-87-03647</t>
+  </si>
+  <si>
+    <t>408-81-22298</t>
+  </si>
+  <si>
+    <t>381-45-00803</t>
+  </si>
+  <si>
+    <t>272-50-00901</t>
+  </si>
+  <si>
+    <t>394-46-00994</t>
+  </si>
+  <si>
+    <t>240-87-02913</t>
+  </si>
+  <si>
+    <t>709-81-03705</t>
+  </si>
+  <si>
+    <t>740-74-00579</t>
+  </si>
+  <si>
+    <t>422-06-00497</t>
+  </si>
+  <si>
+    <t>312-81-80677</t>
+  </si>
+  <si>
+    <t>478-24-01794</t>
+  </si>
+  <si>
+    <t>409-52-00695</t>
+  </si>
+  <si>
+    <t>137-88-03573</t>
+  </si>
+  <si>
+    <t>894-06-00896</t>
+  </si>
+  <si>
+    <t>575-87-02653</t>
+  </si>
+  <si>
+    <t>789-46-00834</t>
+  </si>
+  <si>
+    <t>514-85-28353</t>
+  </si>
+  <si>
+    <t>514-81-63105</t>
+  </si>
+  <si>
+    <t>396-09-02576</t>
+  </si>
+  <si>
+    <t>409-46-12133</t>
+  </si>
+  <si>
+    <t>245-85-01462</t>
+  </si>
+  <si>
+    <t>371-85-01723</t>
+  </si>
+  <si>
+    <t>858-71-00317</t>
+  </si>
+  <si>
+    <t>226-81-37637</t>
+  </si>
+  <si>
+    <t>804-87-03716</t>
+  </si>
+  <si>
+    <t>329-08-03205</t>
+  </si>
+  <si>
+    <t>124-44-05299</t>
+  </si>
+  <si>
+    <t>214-87-42876</t>
+  </si>
+  <si>
+    <t>643-81-03521</t>
+  </si>
+  <si>
+    <t>306-31-21718</t>
+  </si>
+  <si>
+    <t>780-87-03268</t>
+  </si>
+  <si>
+    <t>761-86-03649</t>
+  </si>
+  <si>
+    <t>307-82-03603</t>
+  </si>
+  <si>
+    <t>587-07-03196</t>
+  </si>
+  <si>
+    <t>523-81-01821</t>
+  </si>
+  <si>
+    <t>552-87-01985</t>
+  </si>
+  <si>
+    <t>425-47-00427</t>
+  </si>
+  <si>
+    <t>513-24-02136</t>
+  </si>
+  <si>
+    <t>647-46-00054</t>
+  </si>
+  <si>
+    <t>417-52-00245</t>
+  </si>
+  <si>
+    <t>143-81-12952</t>
+  </si>
+  <si>
+    <t>111-13-35944</t>
+  </si>
+  <si>
+    <t>125-81-85383</t>
+  </si>
+  <si>
+    <t>343-27-01048</t>
+  </si>
+  <si>
+    <t>376-86-01050</t>
+  </si>
+  <si>
+    <t>125-86-18439</t>
+  </si>
+  <si>
+    <t>695-71-00375</t>
+  </si>
+  <si>
+    <t>398-06-03191</t>
+  </si>
+  <si>
+    <t>569-88-01068</t>
+  </si>
+  <si>
+    <t>720-22-02050</t>
+  </si>
+  <si>
+    <t>158-02-02029</t>
+  </si>
+  <si>
+    <t>451-88-01049</t>
+  </si>
+  <si>
+    <t>110-18-69859</t>
+  </si>
+  <si>
+    <t>692-51-00285</t>
+  </si>
+  <si>
+    <t>471-86-00171</t>
+  </si>
+  <si>
+    <t>549-88-03363</t>
+  </si>
+  <si>
+    <t>212-26-36848</t>
+  </si>
+  <si>
+    <t>733-72-00596</t>
+  </si>
+  <si>
+    <t>418-58-00707</t>
   </si>
 </sst>
 </file>
@@ -7418,7 +9017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6138A4-676B-44A6-82D7-1ADA43310F48}">
-  <dimension ref="A1:K282"/>
+  <dimension ref="A1:K343"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -15707,7 +17306,7 @@
         <v>1912</v>
       </c>
     </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="273" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A273" s="32" t="s">
         <v>866</v>
       </c>
@@ -15736,7 +17335,7 @@
         <v>1915</v>
       </c>
     </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="274" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A274" s="32" t="s">
         <v>867</v>
       </c>
@@ -15765,7 +17364,7 @@
         <v>1917</v>
       </c>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="275" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A275" s="32" t="s">
         <v>868</v>
       </c>
@@ -15794,7 +17393,7 @@
         <v>1920</v>
       </c>
     </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="276" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A276" s="32" t="s">
         <v>869</v>
       </c>
@@ -15823,7 +17422,7 @@
         <v>1922</v>
       </c>
     </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="277" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A277" s="32" t="s">
         <v>870</v>
       </c>
@@ -15852,7 +17451,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="278" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A278" s="32" t="s">
         <v>871</v>
       </c>
@@ -15881,7 +17480,7 @@
         <v>1927</v>
       </c>
     </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="279" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A279" s="32" t="s">
         <v>872</v>
       </c>
@@ -15910,7 +17509,7 @@
         <v>1929</v>
       </c>
     </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="280" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A280" s="32" t="s">
         <v>1930</v>
       </c>
@@ -15939,7 +17538,7 @@
         <v>1935</v>
       </c>
     </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="281" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A281" s="32" t="s">
         <v>1938</v>
       </c>
@@ -15968,7 +17567,7 @@
         <v>1944</v>
       </c>
     </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="282" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A282" s="32" t="s">
         <v>1951</v>
       </c>
@@ -15997,16 +17596,1968 @@
         <v>1947</v>
       </c>
     </row>
+    <row r="283" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A283" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B283" t="s">
+        <v>2124</v>
+      </c>
+      <c r="C283" t="s">
+        <v>2125</v>
+      </c>
+      <c r="D283" s="6" t="s">
+        <v>2126</v>
+      </c>
+      <c r="E283" s="6" t="s">
+        <v>2127</v>
+      </c>
+      <c r="F283" s="6" t="s">
+        <v>2128</v>
+      </c>
+      <c r="H283" s="9" t="s">
+        <v>1508</v>
+      </c>
+      <c r="I283" t="s">
+        <v>2129</v>
+      </c>
+      <c r="J283" t="s">
+        <v>280</v>
+      </c>
+      <c r="K283" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="284" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A284" t="s">
+        <v>2597</v>
+      </c>
+      <c r="B284" t="s">
+        <v>2132</v>
+      </c>
+      <c r="C284" t="s">
+        <v>2133</v>
+      </c>
+      <c r="D284" s="6" t="s">
+        <v>2134</v>
+      </c>
+      <c r="E284" s="6" t="s">
+        <v>2135</v>
+      </c>
+      <c r="F284" s="6" t="s">
+        <v>2136</v>
+      </c>
+      <c r="H284" s="9" t="s">
+        <v>2137</v>
+      </c>
+      <c r="I284" t="s">
+        <v>2138</v>
+      </c>
+      <c r="J284" t="s">
+        <v>280</v>
+      </c>
+      <c r="K284" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="285" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A285" t="s">
+        <v>2598</v>
+      </c>
+      <c r="B285" t="s">
+        <v>2139</v>
+      </c>
+      <c r="C285" t="s">
+        <v>2140</v>
+      </c>
+      <c r="D285" s="6" t="s">
+        <v>2141</v>
+      </c>
+      <c r="E285" s="6" t="s">
+        <v>2142</v>
+      </c>
+      <c r="F285" s="6" t="s">
+        <v>2143</v>
+      </c>
+      <c r="H285" s="9" t="s">
+        <v>2144</v>
+      </c>
+      <c r="I285" t="s">
+        <v>2145</v>
+      </c>
+      <c r="J285" t="s">
+        <v>280</v>
+      </c>
+      <c r="K285" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="286" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A286" t="s">
+        <v>2599</v>
+      </c>
+      <c r="B286" t="s">
+        <v>2146</v>
+      </c>
+      <c r="C286" t="s">
+        <v>2147</v>
+      </c>
+      <c r="D286" s="6" t="s">
+        <v>2148</v>
+      </c>
+      <c r="E286" s="6" t="s">
+        <v>2149</v>
+      </c>
+      <c r="F286" s="6" t="s">
+        <v>2150</v>
+      </c>
+      <c r="H286" s="9" t="s">
+        <v>2151</v>
+      </c>
+      <c r="I286" t="s">
+        <v>2152</v>
+      </c>
+      <c r="J286" t="s">
+        <v>2153</v>
+      </c>
+      <c r="K286" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="287" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A287" t="s">
+        <v>2600</v>
+      </c>
+      <c r="B287" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C287" t="s">
+        <v>2156</v>
+      </c>
+      <c r="D287" s="6" t="s">
+        <v>2157</v>
+      </c>
+      <c r="E287" s="6" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F287" s="6" t="s">
+        <v>2159</v>
+      </c>
+      <c r="H287" s="9" t="s">
+        <v>2160</v>
+      </c>
+      <c r="I287" t="s">
+        <v>2161</v>
+      </c>
+      <c r="J287" t="s">
+        <v>280</v>
+      </c>
+      <c r="K287" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="288" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A288" t="s">
+        <v>2601</v>
+      </c>
+      <c r="B288" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C288" t="s">
+        <v>2163</v>
+      </c>
+      <c r="D288" s="6" t="s">
+        <v>2164</v>
+      </c>
+      <c r="E288" s="6" t="s">
+        <v>2165</v>
+      </c>
+      <c r="F288" s="6" t="s">
+        <v>2166</v>
+      </c>
+      <c r="H288" s="9" t="s">
+        <v>2167</v>
+      </c>
+      <c r="I288" t="s">
+        <v>2168</v>
+      </c>
+      <c r="J288" t="s">
+        <v>280</v>
+      </c>
+      <c r="K288" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="289" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A289" t="s">
+        <v>2602</v>
+      </c>
+      <c r="B289" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C289" t="s">
+        <v>2170</v>
+      </c>
+      <c r="D289" s="6" t="s">
+        <v>2171</v>
+      </c>
+      <c r="E289" s="6" t="s">
+        <v>2172</v>
+      </c>
+      <c r="F289" s="6" t="s">
+        <v>2173</v>
+      </c>
+      <c r="H289" s="9" t="s">
+        <v>2174</v>
+      </c>
+      <c r="I289" t="s">
+        <v>2175</v>
+      </c>
+      <c r="J289" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K289" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="290" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A290" t="s">
+        <v>2603</v>
+      </c>
+      <c r="B290" t="s">
+        <v>2178</v>
+      </c>
+      <c r="C290" t="s">
+        <v>2179</v>
+      </c>
+      <c r="D290" s="6" t="s">
+        <v>2180</v>
+      </c>
+      <c r="E290" s="6" t="s">
+        <v>2181</v>
+      </c>
+      <c r="F290" s="6" t="s">
+        <v>2182</v>
+      </c>
+      <c r="H290" s="9" t="s">
+        <v>2183</v>
+      </c>
+      <c r="I290" t="s">
+        <v>2184</v>
+      </c>
+      <c r="J290" t="s">
+        <v>2185</v>
+      </c>
+      <c r="K290" t="s">
+        <v>2186</v>
+      </c>
+    </row>
+    <row r="291" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A291" t="s">
+        <v>2604</v>
+      </c>
+      <c r="B291" t="s">
+        <v>2187</v>
+      </c>
+      <c r="C291" t="s">
+        <v>2188</v>
+      </c>
+      <c r="D291" s="6" t="s">
+        <v>2189</v>
+      </c>
+      <c r="E291" s="6" t="s">
+        <v>2190</v>
+      </c>
+      <c r="F291" s="6" t="s">
+        <v>2191</v>
+      </c>
+      <c r="H291" s="9" t="s">
+        <v>2192</v>
+      </c>
+      <c r="I291" t="s">
+        <v>2193</v>
+      </c>
+      <c r="J291" t="s">
+        <v>2194</v>
+      </c>
+      <c r="K291" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="292" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A292" t="s">
+        <v>2605</v>
+      </c>
+      <c r="B292" t="s">
+        <v>2195</v>
+      </c>
+      <c r="C292" t="s">
+        <v>2196</v>
+      </c>
+      <c r="D292" s="6" t="s">
+        <v>2197</v>
+      </c>
+      <c r="E292" s="6" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F292" s="6" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H292" s="9" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I292" t="s">
+        <v>2201</v>
+      </c>
+      <c r="J292" t="s">
+        <v>280</v>
+      </c>
+      <c r="K292" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="293" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A293" t="s">
+        <v>2606</v>
+      </c>
+      <c r="B293" t="s">
+        <v>2202</v>
+      </c>
+      <c r="C293" t="s">
+        <v>2203</v>
+      </c>
+      <c r="D293" s="6" t="s">
+        <v>2204</v>
+      </c>
+      <c r="E293" s="6" t="s">
+        <v>2205</v>
+      </c>
+      <c r="F293" s="6" t="s">
+        <v>2206</v>
+      </c>
+      <c r="H293" s="9" t="s">
+        <v>2207</v>
+      </c>
+      <c r="I293" t="s">
+        <v>2208</v>
+      </c>
+      <c r="J293" t="s">
+        <v>2209</v>
+      </c>
+      <c r="K293" t="s">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="294" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A294" t="s">
+        <v>2607</v>
+      </c>
+      <c r="B294" t="s">
+        <v>2211</v>
+      </c>
+      <c r="C294" t="s">
+        <v>2212</v>
+      </c>
+      <c r="D294" s="6" t="s">
+        <v>2213</v>
+      </c>
+      <c r="E294" s="6" t="s">
+        <v>2214</v>
+      </c>
+      <c r="F294" s="6" t="s">
+        <v>2215</v>
+      </c>
+      <c r="H294" s="9" t="s">
+        <v>2216</v>
+      </c>
+      <c r="I294" t="s">
+        <v>2217</v>
+      </c>
+      <c r="J294" t="s">
+        <v>2218</v>
+      </c>
+      <c r="K294" t="s">
+        <v>2219</v>
+      </c>
+    </row>
+    <row r="295" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A295" t="s">
+        <v>2608</v>
+      </c>
+      <c r="B295" t="s">
+        <v>2220</v>
+      </c>
+      <c r="C295" t="s">
+        <v>2221</v>
+      </c>
+      <c r="D295" s="6" t="s">
+        <v>2222</v>
+      </c>
+      <c r="E295" s="6" t="s">
+        <v>2223</v>
+      </c>
+      <c r="F295" s="6" t="s">
+        <v>2224</v>
+      </c>
+      <c r="H295" s="9" t="s">
+        <v>2225</v>
+      </c>
+      <c r="I295" t="s">
+        <v>2226</v>
+      </c>
+      <c r="J295" t="s">
+        <v>280</v>
+      </c>
+      <c r="K295" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="296" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A296" t="s">
+        <v>2609</v>
+      </c>
+      <c r="B296" t="s">
+        <v>2227</v>
+      </c>
+      <c r="C296" t="s">
+        <v>2228</v>
+      </c>
+      <c r="D296" s="6" t="s">
+        <v>2229</v>
+      </c>
+      <c r="E296" s="6" t="s">
+        <v>2230</v>
+      </c>
+      <c r="F296" s="6" t="s">
+        <v>2231</v>
+      </c>
+      <c r="H296" s="9" t="s">
+        <v>1453</v>
+      </c>
+      <c r="I296" t="s">
+        <v>2232</v>
+      </c>
+      <c r="J296" t="s">
+        <v>2209</v>
+      </c>
+      <c r="K296" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="297" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A297" t="s">
+        <v>2610</v>
+      </c>
+      <c r="B297" t="s">
+        <v>2233</v>
+      </c>
+      <c r="C297" t="s">
+        <v>2234</v>
+      </c>
+      <c r="D297" s="6" t="s">
+        <v>2235</v>
+      </c>
+      <c r="E297" s="6" t="s">
+        <v>2236</v>
+      </c>
+      <c r="F297" s="6" t="s">
+        <v>2237</v>
+      </c>
+      <c r="H297" s="9" t="s">
+        <v>1635</v>
+      </c>
+      <c r="I297" t="s">
+        <v>2238</v>
+      </c>
+      <c r="J297" t="s">
+        <v>280</v>
+      </c>
+      <c r="K297" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="298" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A298" t="s">
+        <v>2611</v>
+      </c>
+      <c r="B298" t="s">
+        <v>2239</v>
+      </c>
+      <c r="C298" t="s">
+        <v>2240</v>
+      </c>
+      <c r="D298" s="6" t="s">
+        <v>2241</v>
+      </c>
+      <c r="E298" s="6" t="s">
+        <v>2242</v>
+      </c>
+      <c r="F298" s="6" t="s">
+        <v>2243</v>
+      </c>
+      <c r="H298" s="9" t="s">
+        <v>2244</v>
+      </c>
+      <c r="I298" t="s">
+        <v>2245</v>
+      </c>
+      <c r="J298" t="s">
+        <v>2246</v>
+      </c>
+      <c r="K298" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="299" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A299" t="s">
+        <v>2612</v>
+      </c>
+      <c r="B299" t="s">
+        <v>2248</v>
+      </c>
+      <c r="C299" t="s">
+        <v>2249</v>
+      </c>
+      <c r="D299" s="6" t="s">
+        <v>2250</v>
+      </c>
+      <c r="E299" s="6" t="s">
+        <v>2251</v>
+      </c>
+      <c r="F299" s="6" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H299" s="9" t="s">
+        <v>1437</v>
+      </c>
+      <c r="I299" t="s">
+        <v>2253</v>
+      </c>
+      <c r="J299" t="s">
+        <v>2185</v>
+      </c>
+      <c r="K299" t="s">
+        <v>2254</v>
+      </c>
+    </row>
+    <row r="300" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A300" t="s">
+        <v>2613</v>
+      </c>
+      <c r="B300" t="s">
+        <v>2255</v>
+      </c>
+      <c r="C300" t="s">
+        <v>2256</v>
+      </c>
+      <c r="D300" s="6" t="s">
+        <v>2257</v>
+      </c>
+      <c r="E300" s="6" t="s">
+        <v>2258</v>
+      </c>
+      <c r="F300" s="6" t="s">
+        <v>2259</v>
+      </c>
+      <c r="H300" s="9" t="s">
+        <v>2260</v>
+      </c>
+      <c r="I300" t="s">
+        <v>2261</v>
+      </c>
+      <c r="J300" t="s">
+        <v>280</v>
+      </c>
+      <c r="K300" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="301" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A301" t="s">
+        <v>2614</v>
+      </c>
+      <c r="B301" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C301" t="s">
+        <v>2263</v>
+      </c>
+      <c r="D301" s="6" t="s">
+        <v>2264</v>
+      </c>
+      <c r="E301" s="6" t="s">
+        <v>2265</v>
+      </c>
+      <c r="F301" s="6" t="s">
+        <v>2266</v>
+      </c>
+      <c r="H301" s="9" t="s">
+        <v>2267</v>
+      </c>
+      <c r="I301" t="s">
+        <v>2268</v>
+      </c>
+      <c r="J301" t="s">
+        <v>2269</v>
+      </c>
+      <c r="K301" t="s">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="302" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A302" t="s">
+        <v>2615</v>
+      </c>
+      <c r="B302" t="s">
+        <v>2271</v>
+      </c>
+      <c r="C302" t="s">
+        <v>2272</v>
+      </c>
+      <c r="D302" s="6" t="s">
+        <v>2273</v>
+      </c>
+      <c r="E302" s="6" t="s">
+        <v>2274</v>
+      </c>
+      <c r="F302" s="6" t="s">
+        <v>2275</v>
+      </c>
+      <c r="H302" s="9" t="s">
+        <v>2276</v>
+      </c>
+      <c r="I302" t="s">
+        <v>2277</v>
+      </c>
+      <c r="J302" t="s">
+        <v>2278</v>
+      </c>
+      <c r="K302" t="s">
+        <v>2279</v>
+      </c>
+    </row>
+    <row r="303" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A303" t="s">
+        <v>2616</v>
+      </c>
+      <c r="B303" t="s">
+        <v>2280</v>
+      </c>
+      <c r="C303" t="s">
+        <v>2281</v>
+      </c>
+      <c r="D303" s="6" t="s">
+        <v>2282</v>
+      </c>
+      <c r="E303" s="6" t="s">
+        <v>2283</v>
+      </c>
+      <c r="F303" s="6" t="s">
+        <v>2284</v>
+      </c>
+      <c r="H303" s="9" t="s">
+        <v>2285</v>
+      </c>
+      <c r="I303" t="s">
+        <v>2286</v>
+      </c>
+      <c r="J303" t="s">
+        <v>2209</v>
+      </c>
+      <c r="K303" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="304" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A304" t="s">
+        <v>2617</v>
+      </c>
+      <c r="B304" t="s">
+        <v>2287</v>
+      </c>
+      <c r="C304" t="s">
+        <v>2288</v>
+      </c>
+      <c r="D304" s="6" t="s">
+        <v>2289</v>
+      </c>
+      <c r="E304" s="6" t="s">
+        <v>2290</v>
+      </c>
+      <c r="F304" s="6" t="s">
+        <v>2291</v>
+      </c>
+      <c r="H304" s="9" t="s">
+        <v>2292</v>
+      </c>
+      <c r="I304" t="s">
+        <v>2293</v>
+      </c>
+      <c r="J304" t="s">
+        <v>280</v>
+      </c>
+      <c r="K304" t="s">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="305" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A305" t="s">
+        <v>2618</v>
+      </c>
+      <c r="B305" t="s">
+        <v>2295</v>
+      </c>
+      <c r="C305" t="s">
+        <v>2296</v>
+      </c>
+      <c r="D305" s="6" t="s">
+        <v>2297</v>
+      </c>
+      <c r="E305" s="6" t="s">
+        <v>1113</v>
+      </c>
+      <c r="F305" s="6" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H305" s="9" t="s">
+        <v>2298</v>
+      </c>
+      <c r="I305" t="s">
+        <v>2299</v>
+      </c>
+      <c r="J305" t="s">
+        <v>2269</v>
+      </c>
+      <c r="K305" t="s">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="306" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A306" t="s">
+        <v>2619</v>
+      </c>
+      <c r="B306" t="s">
+        <v>2301</v>
+      </c>
+      <c r="C306" t="s">
+        <v>2302</v>
+      </c>
+      <c r="D306" s="6" t="s">
+        <v>2297</v>
+      </c>
+      <c r="E306" s="6" t="s">
+        <v>2303</v>
+      </c>
+      <c r="F306" s="6" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H306" s="9" t="s">
+        <v>2304</v>
+      </c>
+      <c r="I306" t="s">
+        <v>2305</v>
+      </c>
+      <c r="J306" t="s">
+        <v>280</v>
+      </c>
+      <c r="K306" t="s">
+        <v>2306</v>
+      </c>
+    </row>
+    <row r="307" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A307" t="s">
+        <v>2620</v>
+      </c>
+      <c r="B307" t="s">
+        <v>2307</v>
+      </c>
+      <c r="C307" t="s">
+        <v>2308</v>
+      </c>
+      <c r="D307" s="6" t="s">
+        <v>2309</v>
+      </c>
+      <c r="E307" s="6" t="s">
+        <v>2310</v>
+      </c>
+      <c r="F307" s="6" t="s">
+        <v>2311</v>
+      </c>
+      <c r="H307" s="9" t="s">
+        <v>2312</v>
+      </c>
+      <c r="I307" t="s">
+        <v>2313</v>
+      </c>
+      <c r="J307" t="s">
+        <v>2314</v>
+      </c>
+      <c r="K307" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="308" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A308" t="s">
+        <v>2621</v>
+      </c>
+      <c r="B308" t="s">
+        <v>2315</v>
+      </c>
+      <c r="C308" t="s">
+        <v>2316</v>
+      </c>
+      <c r="D308" s="6" t="s">
+        <v>2317</v>
+      </c>
+      <c r="E308" s="6" t="s">
+        <v>2318</v>
+      </c>
+      <c r="F308" s="6" t="s">
+        <v>2319</v>
+      </c>
+      <c r="H308" s="9" t="s">
+        <v>2320</v>
+      </c>
+      <c r="I308" t="s">
+        <v>2321</v>
+      </c>
+      <c r="J308" t="s">
+        <v>2153</v>
+      </c>
+      <c r="K308" t="s">
+        <v>2322</v>
+      </c>
+    </row>
+    <row r="309" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A309" t="s">
+        <v>2622</v>
+      </c>
+      <c r="B309" t="s">
+        <v>2323</v>
+      </c>
+      <c r="C309" t="s">
+        <v>2324</v>
+      </c>
+      <c r="D309" s="6" t="s">
+        <v>2325</v>
+      </c>
+      <c r="E309" s="6" t="s">
+        <v>2326</v>
+      </c>
+      <c r="F309" s="6" t="s">
+        <v>2327</v>
+      </c>
+      <c r="H309" s="9" t="s">
+        <v>1494</v>
+      </c>
+      <c r="I309" t="s">
+        <v>2328</v>
+      </c>
+      <c r="J309" t="s">
+        <v>280</v>
+      </c>
+      <c r="K309" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="310" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A310" t="s">
+        <v>2623</v>
+      </c>
+      <c r="B310" t="s">
+        <v>2330</v>
+      </c>
+      <c r="C310" t="s">
+        <v>2331</v>
+      </c>
+      <c r="D310" s="6" t="s">
+        <v>2332</v>
+      </c>
+      <c r="E310" s="6" t="s">
+        <v>2333</v>
+      </c>
+      <c r="F310" s="6" t="s">
+        <v>2334</v>
+      </c>
+      <c r="H310" s="9" t="s">
+        <v>2335</v>
+      </c>
+      <c r="I310" t="s">
+        <v>2336</v>
+      </c>
+      <c r="J310" t="s">
+        <v>2337</v>
+      </c>
+      <c r="K310" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="311" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A311" t="s">
+        <v>2624</v>
+      </c>
+      <c r="B311" t="s">
+        <v>2338</v>
+      </c>
+      <c r="C311" t="s">
+        <v>2339</v>
+      </c>
+      <c r="D311" s="6" t="s">
+        <v>2340</v>
+      </c>
+      <c r="E311" s="6" t="s">
+        <v>2341</v>
+      </c>
+      <c r="F311" s="6" t="s">
+        <v>2342</v>
+      </c>
+      <c r="H311" s="9" t="s">
+        <v>2343</v>
+      </c>
+      <c r="I311" t="s">
+        <v>2344</v>
+      </c>
+      <c r="J311" t="s">
+        <v>2269</v>
+      </c>
+      <c r="K311" t="s">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="312" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A312" t="s">
+        <v>2625</v>
+      </c>
+      <c r="B312" t="s">
+        <v>2346</v>
+      </c>
+      <c r="C312" t="s">
+        <v>2347</v>
+      </c>
+      <c r="D312" s="6" t="s">
+        <v>2348</v>
+      </c>
+      <c r="E312" s="6" t="s">
+        <v>2349</v>
+      </c>
+      <c r="F312" s="6" t="s">
+        <v>2350</v>
+      </c>
+      <c r="H312" s="9" t="s">
+        <v>2351</v>
+      </c>
+      <c r="I312" t="s">
+        <v>2352</v>
+      </c>
+      <c r="J312" t="s">
+        <v>2246</v>
+      </c>
+      <c r="K312" t="s">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="313" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A313" t="s">
+        <v>2626</v>
+      </c>
+      <c r="B313" t="s">
+        <v>2354</v>
+      </c>
+      <c r="C313" t="s">
+        <v>2355</v>
+      </c>
+      <c r="D313" s="6" t="s">
+        <v>2356</v>
+      </c>
+      <c r="E313" s="6" t="s">
+        <v>2357</v>
+      </c>
+      <c r="F313" s="6" t="s">
+        <v>2358</v>
+      </c>
+      <c r="H313" s="9" t="s">
+        <v>1476</v>
+      </c>
+      <c r="I313" t="s">
+        <v>2359</v>
+      </c>
+      <c r="J313" t="s">
+        <v>280</v>
+      </c>
+      <c r="K313" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="314" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A314" t="s">
+        <v>2627</v>
+      </c>
+      <c r="B314" t="s">
+        <v>2360</v>
+      </c>
+      <c r="C314" t="s">
+        <v>2361</v>
+      </c>
+      <c r="D314" s="6" t="s">
+        <v>2362</v>
+      </c>
+      <c r="E314" s="6" t="s">
+        <v>2363</v>
+      </c>
+      <c r="F314" s="6" t="s">
+        <v>2364</v>
+      </c>
+      <c r="H314" s="9" t="s">
+        <v>2365</v>
+      </c>
+      <c r="I314" t="s">
+        <v>2366</v>
+      </c>
+      <c r="J314" t="s">
+        <v>2367</v>
+      </c>
+      <c r="K314" t="s">
+        <v>2368</v>
+      </c>
+    </row>
+    <row r="315" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A315" t="s">
+        <v>2628</v>
+      </c>
+      <c r="B315" t="s">
+        <v>2369</v>
+      </c>
+      <c r="C315" t="s">
+        <v>2370</v>
+      </c>
+      <c r="D315" s="6" t="s">
+        <v>2371</v>
+      </c>
+      <c r="E315" s="6" t="s">
+        <v>2372</v>
+      </c>
+      <c r="F315" s="6" t="s">
+        <v>2373</v>
+      </c>
+      <c r="H315" s="9" t="s">
+        <v>1577</v>
+      </c>
+      <c r="I315" t="s">
+        <v>2374</v>
+      </c>
+      <c r="J315" t="s">
+        <v>280</v>
+      </c>
+      <c r="K315" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="316" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A316" t="s">
+        <v>2629</v>
+      </c>
+      <c r="B316" t="s">
+        <v>2375</v>
+      </c>
+      <c r="C316" t="s">
+        <v>2376</v>
+      </c>
+      <c r="D316" s="6" t="s">
+        <v>2377</v>
+      </c>
+      <c r="E316" s="6" t="s">
+        <v>2378</v>
+      </c>
+      <c r="F316" s="6" t="s">
+        <v>2379</v>
+      </c>
+      <c r="H316" s="9" t="s">
+        <v>2380</v>
+      </c>
+      <c r="I316" t="s">
+        <v>2381</v>
+      </c>
+      <c r="J316" t="s">
+        <v>280</v>
+      </c>
+      <c r="K316" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="317" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A317" t="s">
+        <v>2630</v>
+      </c>
+      <c r="B317" t="s">
+        <v>2382</v>
+      </c>
+      <c r="C317" t="s">
+        <v>2383</v>
+      </c>
+      <c r="D317" s="6" t="s">
+        <v>2384</v>
+      </c>
+      <c r="E317" s="6" t="s">
+        <v>2385</v>
+      </c>
+      <c r="F317" s="6" t="s">
+        <v>2386</v>
+      </c>
+      <c r="H317" s="9" t="s">
+        <v>2387</v>
+      </c>
+      <c r="I317" t="s">
+        <v>2388</v>
+      </c>
+      <c r="J317" t="s">
+        <v>2389</v>
+      </c>
+      <c r="K317" t="s">
+        <v>2390</v>
+      </c>
+    </row>
+    <row r="318" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A318" t="s">
+        <v>2631</v>
+      </c>
+      <c r="B318" t="s">
+        <v>2391</v>
+      </c>
+      <c r="C318" t="s">
+        <v>2392</v>
+      </c>
+      <c r="D318" s="6" t="s">
+        <v>2393</v>
+      </c>
+      <c r="E318" s="6" t="s">
+        <v>2394</v>
+      </c>
+      <c r="F318" s="6" t="s">
+        <v>2395</v>
+      </c>
+      <c r="H318" s="9" t="s">
+        <v>2396</v>
+      </c>
+      <c r="I318" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J318" t="s">
+        <v>2398</v>
+      </c>
+      <c r="K318" t="s">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="319" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A319" t="s">
+        <v>2632</v>
+      </c>
+      <c r="B319" t="s">
+        <v>2400</v>
+      </c>
+      <c r="C319" t="s">
+        <v>2401</v>
+      </c>
+      <c r="D319" s="6" t="s">
+        <v>2402</v>
+      </c>
+      <c r="E319" s="6" t="s">
+        <v>2403</v>
+      </c>
+      <c r="F319" s="6" t="s">
+        <v>2404</v>
+      </c>
+      <c r="H319" s="9" t="s">
+        <v>2405</v>
+      </c>
+      <c r="I319" t="s">
+        <v>2406</v>
+      </c>
+      <c r="J319" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K319" t="s">
+        <v>2407</v>
+      </c>
+    </row>
+    <row r="320" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A320" t="s">
+        <v>2633</v>
+      </c>
+      <c r="B320" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C320" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D320" s="6" t="s">
+        <v>2410</v>
+      </c>
+      <c r="E320" s="6" t="s">
+        <v>2411</v>
+      </c>
+      <c r="F320" s="6" t="s">
+        <v>2412</v>
+      </c>
+      <c r="H320" s="9" t="s">
+        <v>2413</v>
+      </c>
+      <c r="I320" t="s">
+        <v>2414</v>
+      </c>
+      <c r="J320" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K320" t="s">
+        <v>2415</v>
+      </c>
+    </row>
+    <row r="321" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A321" t="s">
+        <v>2634</v>
+      </c>
+      <c r="B321" t="s">
+        <v>2416</v>
+      </c>
+      <c r="C321" t="s">
+        <v>2417</v>
+      </c>
+      <c r="D321" s="6" t="s">
+        <v>2418</v>
+      </c>
+      <c r="E321" s="6" t="s">
+        <v>2419</v>
+      </c>
+      <c r="F321" s="6" t="s">
+        <v>2420</v>
+      </c>
+      <c r="H321" s="9" t="s">
+        <v>2421</v>
+      </c>
+      <c r="I321" t="s">
+        <v>2422</v>
+      </c>
+      <c r="J321" t="s">
+        <v>2423</v>
+      </c>
+      <c r="K321" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="322" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A322" t="s">
+        <v>2635</v>
+      </c>
+      <c r="B322" t="s">
+        <v>2424</v>
+      </c>
+      <c r="C322" t="s">
+        <v>2425</v>
+      </c>
+      <c r="D322" s="6" t="s">
+        <v>2426</v>
+      </c>
+      <c r="E322" s="6" t="s">
+        <v>2427</v>
+      </c>
+      <c r="F322" s="6" t="s">
+        <v>2428</v>
+      </c>
+      <c r="H322" s="9" t="s">
+        <v>2429</v>
+      </c>
+      <c r="I322" t="s">
+        <v>2430</v>
+      </c>
+      <c r="J322" t="s">
+        <v>280</v>
+      </c>
+      <c r="K322" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="323" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A323" t="s">
+        <v>2636</v>
+      </c>
+      <c r="B323" t="s">
+        <v>2431</v>
+      </c>
+      <c r="C323" t="s">
+        <v>2432</v>
+      </c>
+      <c r="D323" s="6" t="s">
+        <v>2433</v>
+      </c>
+      <c r="E323" s="6" t="s">
+        <v>2434</v>
+      </c>
+      <c r="F323" s="6" t="s">
+        <v>2435</v>
+      </c>
+      <c r="H323" s="9" t="s">
+        <v>2436</v>
+      </c>
+      <c r="I323" t="s">
+        <v>2437</v>
+      </c>
+      <c r="J323" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K323" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="324" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A324" t="s">
+        <v>2637</v>
+      </c>
+      <c r="B324" t="s">
+        <v>2440</v>
+      </c>
+      <c r="C324" t="s">
+        <v>2441</v>
+      </c>
+      <c r="D324" s="6" t="s">
+        <v>2442</v>
+      </c>
+      <c r="E324" s="6" t="s">
+        <v>2443</v>
+      </c>
+      <c r="F324" s="6" t="s">
+        <v>2444</v>
+      </c>
+      <c r="H324" s="9" t="s">
+        <v>2445</v>
+      </c>
+      <c r="I324" t="s">
+        <v>2446</v>
+      </c>
+      <c r="J324" t="s">
+        <v>280</v>
+      </c>
+      <c r="K324" t="s">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="325" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A325" t="s">
+        <v>2638</v>
+      </c>
+      <c r="B325" t="s">
+        <v>2447</v>
+      </c>
+      <c r="C325" t="s">
+        <v>2448</v>
+      </c>
+      <c r="D325" s="6" t="s">
+        <v>2449</v>
+      </c>
+      <c r="E325" s="6" t="s">
+        <v>2450</v>
+      </c>
+      <c r="F325" s="6" t="s">
+        <v>2451</v>
+      </c>
+      <c r="H325" s="9" t="s">
+        <v>2452</v>
+      </c>
+      <c r="I325" t="s">
+        <v>2453</v>
+      </c>
+      <c r="J325" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K325" t="s">
+        <v>2454</v>
+      </c>
+    </row>
+    <row r="326" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A326" t="s">
+        <v>2639</v>
+      </c>
+      <c r="B326" t="s">
+        <v>2455</v>
+      </c>
+      <c r="C326" t="s">
+        <v>2456</v>
+      </c>
+      <c r="D326" s="6" t="s">
+        <v>2457</v>
+      </c>
+      <c r="E326" s="6" t="s">
+        <v>2458</v>
+      </c>
+      <c r="F326" s="6" t="s">
+        <v>2459</v>
+      </c>
+      <c r="H326" s="9" t="s">
+        <v>2460</v>
+      </c>
+      <c r="I326" t="s">
+        <v>2461</v>
+      </c>
+      <c r="J326" t="s">
+        <v>280</v>
+      </c>
+      <c r="K326" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="327" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A327" t="s">
+        <v>2640</v>
+      </c>
+      <c r="B327" t="s">
+        <v>2462</v>
+      </c>
+      <c r="C327" t="s">
+        <v>2463</v>
+      </c>
+      <c r="D327" s="6" t="s">
+        <v>2464</v>
+      </c>
+      <c r="E327" s="6" t="s">
+        <v>2465</v>
+      </c>
+      <c r="F327" s="6" t="s">
+        <v>2466</v>
+      </c>
+      <c r="H327" s="9" t="s">
+        <v>2467</v>
+      </c>
+      <c r="I327" t="s">
+        <v>2468</v>
+      </c>
+      <c r="J327" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K327" t="s">
+        <v>2469</v>
+      </c>
+    </row>
+    <row r="328" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A328" t="s">
+        <v>2641</v>
+      </c>
+      <c r="B328" t="s">
+        <v>2470</v>
+      </c>
+      <c r="C328" t="s">
+        <v>2471</v>
+      </c>
+      <c r="D328" s="6" t="s">
+        <v>2472</v>
+      </c>
+      <c r="E328" s="6" t="s">
+        <v>2473</v>
+      </c>
+      <c r="F328" s="6" t="s">
+        <v>2474</v>
+      </c>
+      <c r="H328" s="9" t="s">
+        <v>2475</v>
+      </c>
+      <c r="I328" t="s">
+        <v>2476</v>
+      </c>
+      <c r="J328" t="s">
+        <v>280</v>
+      </c>
+      <c r="K328" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="329" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A329" t="s">
+        <v>2642</v>
+      </c>
+      <c r="B329" t="s">
+        <v>2477</v>
+      </c>
+      <c r="C329" t="s">
+        <v>2478</v>
+      </c>
+      <c r="D329" s="6" t="s">
+        <v>2479</v>
+      </c>
+      <c r="E329" s="6" t="s">
+        <v>2480</v>
+      </c>
+      <c r="F329" s="6" t="s">
+        <v>2481</v>
+      </c>
+      <c r="H329" s="9" t="s">
+        <v>2482</v>
+      </c>
+      <c r="I329" t="s">
+        <v>2483</v>
+      </c>
+      <c r="J329" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K329" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="330" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A330" t="s">
+        <v>2643</v>
+      </c>
+      <c r="B330" t="s">
+        <v>2485</v>
+      </c>
+      <c r="C330" t="s">
+        <v>2486</v>
+      </c>
+      <c r="D330" s="6" t="s">
+        <v>2487</v>
+      </c>
+      <c r="E330" s="6" t="s">
+        <v>2488</v>
+      </c>
+      <c r="F330" s="6" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H330" s="9" t="s">
+        <v>2489</v>
+      </c>
+      <c r="I330" t="s">
+        <v>2490</v>
+      </c>
+      <c r="J330" t="s">
+        <v>2269</v>
+      </c>
+      <c r="K330" t="s">
+        <v>2491</v>
+      </c>
+    </row>
+    <row r="331" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A331" t="s">
+        <v>2644</v>
+      </c>
+      <c r="B331" t="s">
+        <v>2492</v>
+      </c>
+      <c r="C331" t="s">
+        <v>2493</v>
+      </c>
+      <c r="D331" s="6" t="s">
+        <v>2494</v>
+      </c>
+      <c r="E331" s="6" t="s">
+        <v>2495</v>
+      </c>
+      <c r="F331" s="6" t="s">
+        <v>2496</v>
+      </c>
+      <c r="H331" s="9" t="s">
+        <v>2497</v>
+      </c>
+      <c r="I331" t="s">
+        <v>2498</v>
+      </c>
+      <c r="J331" t="s">
+        <v>2499</v>
+      </c>
+      <c r="K331" t="s">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="332" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A332" t="s">
+        <v>2645</v>
+      </c>
+      <c r="B332" t="s">
+        <v>2501</v>
+      </c>
+      <c r="C332" t="s">
+        <v>2502</v>
+      </c>
+      <c r="D332" s="6" t="s">
+        <v>2503</v>
+      </c>
+      <c r="E332" s="6" t="s">
+        <v>2504</v>
+      </c>
+      <c r="F332" s="6" t="s">
+        <v>2505</v>
+      </c>
+      <c r="H332" s="9" t="s">
+        <v>2506</v>
+      </c>
+      <c r="I332" t="s">
+        <v>2507</v>
+      </c>
+      <c r="J332" t="s">
+        <v>280</v>
+      </c>
+      <c r="K332" t="s">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="333" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A333" t="s">
+        <v>2646</v>
+      </c>
+      <c r="B333" t="s">
+        <v>2508</v>
+      </c>
+      <c r="C333" t="s">
+        <v>2509</v>
+      </c>
+      <c r="D333" s="6" t="s">
+        <v>2510</v>
+      </c>
+      <c r="E333" s="6" t="s">
+        <v>2511</v>
+      </c>
+      <c r="F333" s="6" t="s">
+        <v>2512</v>
+      </c>
+      <c r="H333" s="9" t="s">
+        <v>2513</v>
+      </c>
+      <c r="I333" t="s">
+        <v>2514</v>
+      </c>
+      <c r="J333" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K333" t="s">
+        <v>2515</v>
+      </c>
+    </row>
+    <row r="334" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A334" t="s">
+        <v>2647</v>
+      </c>
+      <c r="B334" t="s">
+        <v>2516</v>
+      </c>
+      <c r="C334" t="s">
+        <v>2517</v>
+      </c>
+      <c r="D334" s="6" t="s">
+        <v>2518</v>
+      </c>
+      <c r="E334" s="6" t="s">
+        <v>2519</v>
+      </c>
+      <c r="F334" s="6" t="s">
+        <v>2520</v>
+      </c>
+      <c r="H334" s="9" t="s">
+        <v>2521</v>
+      </c>
+      <c r="I334" t="s">
+        <v>2522</v>
+      </c>
+      <c r="J334" t="s">
+        <v>2523</v>
+      </c>
+      <c r="K334" t="s">
+        <v>2524</v>
+      </c>
+    </row>
+    <row r="335" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A335" t="s">
+        <v>2648</v>
+      </c>
+      <c r="B335" t="s">
+        <v>2525</v>
+      </c>
+      <c r="C335" t="s">
+        <v>2526</v>
+      </c>
+      <c r="D335" s="6" t="s">
+        <v>2527</v>
+      </c>
+      <c r="E335" s="6" t="s">
+        <v>2528</v>
+      </c>
+      <c r="F335" s="6" t="s">
+        <v>2529</v>
+      </c>
+      <c r="H335" s="9" t="s">
+        <v>2530</v>
+      </c>
+      <c r="I335" t="s">
+        <v>2531</v>
+      </c>
+      <c r="J335" t="s">
+        <v>2523</v>
+      </c>
+      <c r="K335" t="s">
+        <v>2532</v>
+      </c>
+    </row>
+    <row r="336" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A336" t="s">
+        <v>2649</v>
+      </c>
+      <c r="B336" t="s">
+        <v>2533</v>
+      </c>
+      <c r="C336" t="s">
+        <v>2534</v>
+      </c>
+      <c r="D336" s="6" t="s">
+        <v>2535</v>
+      </c>
+      <c r="E336" s="6" t="s">
+        <v>2536</v>
+      </c>
+      <c r="F336" s="6" t="s">
+        <v>2537</v>
+      </c>
+      <c r="H336" s="9" t="s">
+        <v>2538</v>
+      </c>
+      <c r="I336" t="s">
+        <v>2539</v>
+      </c>
+      <c r="J336" t="s">
+        <v>2423</v>
+      </c>
+      <c r="K336" t="s">
+        <v>2540</v>
+      </c>
+    </row>
+    <row r="337" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A337" t="s">
+        <v>2650</v>
+      </c>
+      <c r="B337" t="s">
+        <v>2541</v>
+      </c>
+      <c r="C337" t="s">
+        <v>2542</v>
+      </c>
+      <c r="D337" s="6" t="s">
+        <v>2543</v>
+      </c>
+      <c r="E337" s="6" t="s">
+        <v>2544</v>
+      </c>
+      <c r="F337" s="6" t="s">
+        <v>2545</v>
+      </c>
+      <c r="H337" s="9" t="s">
+        <v>2546</v>
+      </c>
+      <c r="I337" t="s">
+        <v>2547</v>
+      </c>
+      <c r="J337" t="s">
+        <v>2548</v>
+      </c>
+      <c r="K337" t="s">
+        <v>2549</v>
+      </c>
+    </row>
+    <row r="338" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A338" t="s">
+        <v>2651</v>
+      </c>
+      <c r="B338" t="s">
+        <v>2550</v>
+      </c>
+      <c r="C338" t="s">
+        <v>2551</v>
+      </c>
+      <c r="D338" s="6" t="s">
+        <v>2552</v>
+      </c>
+      <c r="E338" s="6" t="s">
+        <v>2553</v>
+      </c>
+      <c r="F338" s="6" t="s">
+        <v>2554</v>
+      </c>
+      <c r="H338" s="9" t="s">
+        <v>2555</v>
+      </c>
+      <c r="I338" t="s">
+        <v>2556</v>
+      </c>
+      <c r="J338" t="s">
+        <v>2423</v>
+      </c>
+      <c r="K338" t="s">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="339" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A339" t="s">
+        <v>2652</v>
+      </c>
+      <c r="B339" t="s">
+        <v>2557</v>
+      </c>
+      <c r="C339" t="s">
+        <v>2558</v>
+      </c>
+      <c r="D339" s="6" t="s">
+        <v>2559</v>
+      </c>
+      <c r="E339" s="6" t="s">
+        <v>2560</v>
+      </c>
+      <c r="F339" s="6" t="s">
+        <v>2561</v>
+      </c>
+      <c r="H339" s="9" t="s">
+        <v>2562</v>
+      </c>
+      <c r="I339" t="s">
+        <v>2563</v>
+      </c>
+      <c r="J339" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K339" t="s">
+        <v>2564</v>
+      </c>
+    </row>
+    <row r="340" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A340" t="s">
+        <v>2653</v>
+      </c>
+      <c r="B340" t="s">
+        <v>2565</v>
+      </c>
+      <c r="C340" t="s">
+        <v>2566</v>
+      </c>
+      <c r="D340" s="6" t="s">
+        <v>2567</v>
+      </c>
+      <c r="E340" s="6" t="s">
+        <v>2568</v>
+      </c>
+      <c r="F340" s="6" t="s">
+        <v>2569</v>
+      </c>
+      <c r="H340" s="9" t="s">
+        <v>2570</v>
+      </c>
+      <c r="I340" t="s">
+        <v>2571</v>
+      </c>
+      <c r="J340" t="s">
+        <v>280</v>
+      </c>
+      <c r="K340" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="341" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A341" t="s">
+        <v>2654</v>
+      </c>
+      <c r="B341" t="s">
+        <v>2572</v>
+      </c>
+      <c r="C341" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D341" s="6" t="s">
+        <v>2574</v>
+      </c>
+      <c r="E341" s="6" t="s">
+        <v>2575</v>
+      </c>
+      <c r="F341" s="6" t="s">
+        <v>2576</v>
+      </c>
+      <c r="H341" s="9" t="s">
+        <v>2577</v>
+      </c>
+      <c r="I341" t="s">
+        <v>2578</v>
+      </c>
+      <c r="J341" t="s">
+        <v>284</v>
+      </c>
+      <c r="K341" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="342" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A342" t="s">
+        <v>2655</v>
+      </c>
+      <c r="B342" t="s">
+        <v>2579</v>
+      </c>
+      <c r="C342" t="s">
+        <v>2580</v>
+      </c>
+      <c r="D342" s="6" t="s">
+        <v>2581</v>
+      </c>
+      <c r="E342" s="6" t="s">
+        <v>2582</v>
+      </c>
+      <c r="F342" s="6" t="s">
+        <v>2583</v>
+      </c>
+      <c r="H342" s="9" t="s">
+        <v>2584</v>
+      </c>
+      <c r="I342" t="s">
+        <v>2585</v>
+      </c>
+      <c r="J342" t="s">
+        <v>2586</v>
+      </c>
+      <c r="K342" t="s">
+        <v>2587</v>
+      </c>
+    </row>
+    <row r="343" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A343" t="s">
+        <v>2656</v>
+      </c>
+      <c r="B343" t="s">
+        <v>2588</v>
+      </c>
+      <c r="C343" t="s">
+        <v>2589</v>
+      </c>
+      <c r="D343" s="6" t="s">
+        <v>2590</v>
+      </c>
+      <c r="E343" s="6" t="s">
+        <v>2591</v>
+      </c>
+      <c r="F343" s="6" t="s">
+        <v>2592</v>
+      </c>
+      <c r="H343" s="9" t="s">
+        <v>2593</v>
+      </c>
+      <c r="I343" t="s">
+        <v>2594</v>
+      </c>
+      <c r="J343" t="s">
+        <v>280</v>
+      </c>
+      <c r="K343" t="s">
+        <v>2595</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A1:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>